<commit_message>
add new envoices  and moove old invoices to old_full envoices folder
</commit_message>
<xml_diff>
--- a/Chadwicks_FULL_INVOICES_TEST_NO_MATERIAL.xlsx
+++ b/Chadwicks_FULL_INVOICES_TEST_NO_MATERIAL.xlsx
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J180"/>
+  <dimension ref="A1:J182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="J2" s="7" t="n">
-        <v>46281.4403702179</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="3">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>46281.44037021817</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="4">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="J4" s="7" t="n">
-        <v>46281.44037021828</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="5">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>46281.44037021837</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="6">
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>46281.44037021845</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>46281.44037021854</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="8">
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>46281.44037021863</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="9">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>46281.4403702187</v>
+        <v>46281.44037021991</v>
       </c>
     </row>
     <row r="10">
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="J10" s="7" t="n">
-        <v>46281.44045687889</v>
+        <v>46281.440456875</v>
       </c>
     </row>
     <row r="11">
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="J11" s="7" t="n">
-        <v>46281.44037319587</v>
+        <v>46281.44037319445</v>
       </c>
     </row>
     <row r="12">
@@ -1020,7 +1020,7 @@
         </is>
       </c>
       <c r="J12" s="7" t="n">
-        <v>46281.44037319559</v>
+        <v>46281.44037319445</v>
       </c>
     </row>
     <row r="13">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>46281.44045687928</v>
+        <v>46281.440456875</v>
       </c>
     </row>
     <row r="14">
@@ -1096,7 +1096,7 @@
         </is>
       </c>
       <c r="J14" s="7" t="n">
-        <v>46281.44044909765</v>
+        <v>46281.44044909722</v>
       </c>
     </row>
     <row r="15">
@@ -1138,7 +1138,7 @@
         </is>
       </c>
       <c r="J15" s="7" t="n">
-        <v>46281.44037534914</v>
+        <v>46281.44037534722</v>
       </c>
     </row>
     <row r="16">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="J16" s="7" t="n">
-        <v>46281.44037534983</v>
+        <v>46281.44037534722</v>
       </c>
     </row>
     <row r="17">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="J17" s="7" t="n">
-        <v>46281.44037641572</v>
+        <v>46281.44037641204</v>
       </c>
     </row>
     <row r="18">
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>46281.44037641602</v>
+        <v>46281.44037641204</v>
       </c>
     </row>
     <row r="19">
@@ -1282,7 +1282,7 @@
         </is>
       </c>
       <c r="J19" s="7" t="n">
-        <v>46281.44037641613</v>
+        <v>46281.44037641204</v>
       </c>
     </row>
     <row r="20">
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="J20" s="7" t="n">
-        <v>46281.44038170587</v>
+        <v>46281.44038170139</v>
       </c>
     </row>
     <row r="21">
@@ -1350,7 +1350,7 @@
         </is>
       </c>
       <c r="J21" s="7" t="n">
-        <v>46281.44038170621</v>
+        <v>46281.44038170139</v>
       </c>
     </row>
     <row r="22">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>46281.44038170633</v>
+        <v>46281.44038170139</v>
       </c>
     </row>
     <row r="23">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="J23" s="7" t="n">
-        <v>46281.44045966078</v>
+        <v>46281.53116448341</v>
       </c>
     </row>
     <row r="24">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="J24" s="7" t="n">
-        <v>46281.44045966106</v>
+        <v>46281.53116448369</v>
       </c>
     </row>
     <row r="25">
@@ -1498,11 +1498,11 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>SX235981</t>
+          <t>SX236219</t>
         </is>
       </c>
       <c r="J25" s="7" t="n">
-        <v>46281.44045966119</v>
+        <v>46281.53116769179</v>
       </c>
     </row>
     <row r="26">
@@ -1540,11 +1540,11 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>SX235645</t>
+          <t>SX236219</t>
         </is>
       </c>
       <c r="J26" s="7" t="n">
-        <v>46281.4404521908</v>
+        <v>46281.53116769207</v>
       </c>
     </row>
     <row r="27">
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>46281.44045219098</v>
+        <v>46281.4404521875</v>
       </c>
     </row>
     <row r="28">
@@ -1616,11 +1616,11 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>SX235645</t>
+          <t>SX236219</t>
         </is>
       </c>
       <c r="J28" s="7" t="n">
-        <v>46281.44045219109</v>
+        <v>46281.53116769218</v>
       </c>
     </row>
     <row r="29">
@@ -1650,11 +1650,11 @@
       <c r="H29" s="6" t="n"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SX235981</t>
+          <t>SX236219</t>
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>46281.44045966139</v>
+        <v>46281.53116769236</v>
       </c>
     </row>
     <row r="30">
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="J30" s="7" t="n">
-        <v>46281.44040841375</v>
+        <v>46281.44040841435</v>
       </c>
     </row>
     <row r="31">
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="J31" s="7" t="n">
-        <v>46281.44040841402</v>
+        <v>46281.44040841435</v>
       </c>
     </row>
     <row r="32">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="J32" s="7" t="n">
-        <v>46281.44040930187</v>
+        <v>46281.44040930556</v>
       </c>
     </row>
     <row r="33">
@@ -1798,7 +1798,7 @@
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>46281.44045779933</v>
+        <v>46281.44045780093</v>
       </c>
     </row>
     <row r="34">
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="J34" s="7" t="n">
-        <v>46281.44041546599</v>
+        <v>46281.44041546297</v>
       </c>
     </row>
     <row r="35">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="J35" s="7" t="n">
-        <v>46281.44042378209</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="36">
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="J36" s="7" t="n">
-        <v>46281.44042378237</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="37">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="J37" s="7" t="n">
-        <v>46281.440425774</v>
+        <v>46281.44042577546</v>
       </c>
     </row>
     <row r="38">
@@ -1984,7 +1984,7 @@
         </is>
       </c>
       <c r="J38" s="7" t="n">
-        <v>46281.44042378295</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="39">
@@ -2018,7 +2018,7 @@
         </is>
       </c>
       <c r="J39" s="7" t="n">
-        <v>46281.44042378305</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="40">
@@ -2052,7 +2052,7 @@
         </is>
       </c>
       <c r="J40" s="7" t="n">
-        <v>46281.44042378313</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="41">
@@ -2086,7 +2086,7 @@
         </is>
       </c>
       <c r="J41" s="7" t="n">
-        <v>46281.44042378321</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="42">
@@ -2120,7 +2120,7 @@
         </is>
       </c>
       <c r="J42" s="7" t="n">
-        <v>46281.44042378329</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="43">
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="J43" s="7" t="n">
-        <v>46281.44042378337</v>
+        <v>46281.44042378472</v>
       </c>
     </row>
     <row r="44">
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="J44" s="7" t="n">
-        <v>46281.44045094141</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="45">
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="J45" s="7" t="n">
-        <v>46281.44045219089</v>
+        <v>46281.4404521875</v>
       </c>
     </row>
     <row r="46">
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="J46" s="7" t="n">
-        <v>46281.44042577352</v>
+        <v>46281.44042577546</v>
       </c>
     </row>
     <row r="47">
@@ -2298,7 +2298,7 @@
         </is>
       </c>
       <c r="J47" s="7" t="n">
-        <v>46281.44042577377</v>
+        <v>46281.44042577546</v>
       </c>
     </row>
     <row r="48">
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="J48" s="7" t="n">
-        <v>46281.44042577389</v>
+        <v>46281.44042577546</v>
       </c>
     </row>
     <row r="49">
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="J49" s="7" t="n">
-        <v>46281.44042673074</v>
+        <v>46281.44042673611</v>
       </c>
     </row>
     <row r="50">
@@ -2400,7 +2400,7 @@
         </is>
       </c>
       <c r="J50" s="7" t="n">
-        <v>46281.44045094048</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="51">
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="J51" s="7" t="n">
-        <v>46281.44042764218</v>
+        <v>46281.44042763889</v>
       </c>
     </row>
     <row r="52">
@@ -2472,11 +2472,11 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>SX234913</t>
+          <t>SX236219</t>
         </is>
       </c>
       <c r="J52" s="7" t="n">
-        <v>46281.44044117114</v>
+        <v>46281.53116769227</v>
       </c>
     </row>
     <row r="53">
@@ -2510,7 +2510,7 @@
         </is>
       </c>
       <c r="J53" s="7" t="n">
-        <v>46281.4404462991</v>
+        <v>46281.4404462963</v>
       </c>
     </row>
     <row r="54">
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="J54" s="7" t="n">
-        <v>46281.44043687537</v>
+        <v>46281.440436875</v>
       </c>
     </row>
     <row r="55">
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="J55" s="7" t="n">
-        <v>46281.44044629885</v>
+        <v>46281.4404462963</v>
       </c>
     </row>
     <row r="56">
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J56" s="7" t="n">
-        <v>46281.44043687582</v>
+        <v>46281.440436875</v>
       </c>
     </row>
     <row r="57">
@@ -2654,7 +2654,7 @@
         </is>
       </c>
       <c r="J57" s="7" t="n">
-        <v>46281.44045966129</v>
+        <v>46281.53116448391</v>
       </c>
     </row>
     <row r="58">
@@ -2688,7 +2688,7 @@
         </is>
       </c>
       <c r="J58" s="7" t="n">
-        <v>46281.44045687938</v>
+        <v>46281.440456875</v>
       </c>
     </row>
     <row r="59">
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="J59" s="7" t="n">
-        <v>46281.44043790585</v>
+        <v>46281.44043790509</v>
       </c>
     </row>
     <row r="60">
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="J60" s="7" t="n">
-        <v>46281.44044000062</v>
+        <v>46281.44044</v>
       </c>
     </row>
     <row r="61">
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="J61" s="7" t="n">
-        <v>46281.44043790615</v>
+        <v>46281.44043790509</v>
       </c>
     </row>
     <row r="62">
@@ -2824,7 +2824,7 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>46281.44043892811</v>
+        <v>46281.44043892361</v>
       </c>
     </row>
     <row r="63">
@@ -2858,7 +2858,7 @@
         </is>
       </c>
       <c r="J63" s="7" t="n">
-        <v>46281.44043999979</v>
+        <v>46281.44044</v>
       </c>
     </row>
     <row r="64">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="J64" s="7" t="n">
-        <v>46281.44044000011</v>
+        <v>46281.44044</v>
       </c>
     </row>
     <row r="65">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="J65" s="7" t="n">
-        <v>46281.44044000025</v>
+        <v>46281.44044</v>
       </c>
     </row>
     <row r="66">
@@ -2960,7 +2960,7 @@
         </is>
       </c>
       <c r="J66" s="7" t="n">
-        <v>46281.44044000035</v>
+        <v>46281.44044</v>
       </c>
     </row>
     <row r="67">
@@ -2994,7 +2994,7 @@
         </is>
       </c>
       <c r="J67" s="7" t="n">
-        <v>46281.44044000044</v>
+        <v>46281.44044</v>
       </c>
     </row>
     <row r="68">
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="J68" s="7" t="n">
-        <v>46281.44044000053</v>
+        <v>46281.44044</v>
       </c>
     </row>
     <row r="69">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="J69" s="7" t="n">
-        <v>46281.44044335377</v>
+        <v>46281.44044335649</v>
       </c>
     </row>
     <row r="70">
@@ -3096,7 +3096,7 @@
         </is>
       </c>
       <c r="J70" s="7" t="n">
-        <v>46281.44044335408</v>
+        <v>46281.44044335649</v>
       </c>
     </row>
     <row r="71">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="J71" s="7" t="n">
-        <v>46281.44044722117</v>
+        <v>46281.44044722222</v>
       </c>
     </row>
     <row r="72">
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="J72" s="7" t="n">
-        <v>46281.44044722156</v>
+        <v>46281.44044722222</v>
       </c>
     </row>
     <row r="73">
@@ -3198,7 +3198,7 @@
         </is>
       </c>
       <c r="J73" s="7" t="n">
-        <v>46281.44044722172</v>
+        <v>46281.44044722222</v>
       </c>
     </row>
     <row r="74">
@@ -3232,7 +3232,7 @@
         </is>
       </c>
       <c r="J74" s="7" t="n">
-        <v>46281.44044812881</v>
+        <v>46281.440448125</v>
       </c>
     </row>
     <row r="75">
@@ -3266,7 +3266,7 @@
         </is>
       </c>
       <c r="J75" s="7" t="n">
-        <v>46281.44044812919</v>
+        <v>46281.440448125</v>
       </c>
     </row>
     <row r="76">
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="J76" s="7" t="n">
-        <v>46281.44044909726</v>
+        <v>46281.44044909722</v>
       </c>
     </row>
     <row r="77">
@@ -3334,7 +3334,7 @@
         </is>
       </c>
       <c r="J77" s="7" t="n">
-        <v>46281.44044909752</v>
+        <v>46281.44044909722</v>
       </c>
     </row>
     <row r="78">
@@ -3368,7 +3368,7 @@
         </is>
       </c>
       <c r="J78" s="7" t="n">
-        <v>46281.44045094008</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="79">
@@ -3402,7 +3402,7 @@
         </is>
       </c>
       <c r="J79" s="7" t="n">
-        <v>46281.44045094035</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="80">
@@ -3436,7 +3436,7 @@
         </is>
       </c>
       <c r="J80" s="7" t="n">
-        <v>46281.4404509406</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="81">
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>46281.4404509407</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="82">
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="J82" s="7" t="n">
-        <v>46281.44045094079</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="83">
@@ -3538,7 +3538,7 @@
         </is>
       </c>
       <c r="J83" s="7" t="n">
-        <v>46281.44045094087</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="84">
@@ -3572,7 +3572,7 @@
         </is>
       </c>
       <c r="J84" s="7" t="n">
-        <v>46281.44045094097</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="85">
@@ -3606,7 +3606,7 @@
         </is>
       </c>
       <c r="J85" s="7" t="n">
-        <v>46281.44045094107</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="86">
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="J86" s="7" t="n">
-        <v>46281.44045094123</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="87">
@@ -3674,7 +3674,7 @@
         </is>
       </c>
       <c r="J87" s="7" t="n">
-        <v>46281.44045094132</v>
+        <v>46281.4404509375</v>
       </c>
     </row>
     <row r="88">
@@ -3708,7 +3708,7 @@
         </is>
       </c>
       <c r="J88" s="7" t="n">
-        <v>46281.44045400789</v>
+        <v>46281.44045400463</v>
       </c>
     </row>
     <row r="89">
@@ -3742,7 +3742,7 @@
         </is>
       </c>
       <c r="J89" s="7" t="n">
-        <v>46281.44045400817</v>
+        <v>46281.44045400463</v>
       </c>
     </row>
     <row r="90">
@@ -3776,7 +3776,7 @@
         </is>
       </c>
       <c r="J90" s="7" t="n">
-        <v>46281.44045491649</v>
+        <v>46281.44045491898</v>
       </c>
     </row>
     <row r="91">
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="J91" s="7" t="n">
-        <v>46281.44045593853</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="92">
@@ -3844,7 +3844,7 @@
         </is>
       </c>
       <c r="J92" s="7" t="n">
-        <v>46281.4404559388</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="93">
@@ -3878,7 +3878,7 @@
         </is>
       </c>
       <c r="J93" s="7" t="n">
-        <v>46281.4404559389</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="94">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="J94" s="7" t="n">
-        <v>46281.440455939</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="95">
@@ -3946,7 +3946,7 @@
         </is>
       </c>
       <c r="J95" s="7" t="n">
-        <v>46281.4404559391</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="96">
@@ -3980,7 +3980,7 @@
         </is>
       </c>
       <c r="J96" s="7" t="n">
-        <v>46281.44045593919</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="97">
@@ -4014,7 +4014,7 @@
         </is>
       </c>
       <c r="J97" s="7" t="n">
-        <v>46281.44045593927</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="98">
@@ -4048,7 +4048,7 @@
         </is>
       </c>
       <c r="J98" s="7" t="n">
-        <v>46281.44045593937</v>
+        <v>46281.4404559375</v>
       </c>
     </row>
     <row r="99">
@@ -4078,11 +4078,11 @@
       <c r="H99" s="6" t="n"/>
       <c r="I99" t="inlineStr">
         <is>
-          <t>SX235828</t>
+          <t>CA316114</t>
         </is>
       </c>
       <c r="J99" s="7" t="n">
-        <v>46281.44045687917</v>
+        <v>46281.53116159909</v>
       </c>
     </row>
     <row r="100">
@@ -4116,7 +4116,7 @@
         </is>
       </c>
       <c r="J100" s="7" t="n">
-        <v>46281.44045868923</v>
+        <v>46281.53116347721</v>
       </c>
     </row>
     <row r="101">
@@ -4150,7 +4150,7 @@
         </is>
       </c>
       <c r="J101" s="7" t="n">
-        <v>46281.4404605484</v>
+        <v>46281.53116544029</v>
       </c>
     </row>
     <row r="102">
@@ -4184,7 +4184,7 @@
         </is>
       </c>
       <c r="J102" s="7" t="n">
-        <v>46281.44036814972</v>
+        <v>46281.44036814815</v>
       </c>
     </row>
     <row r="103">
@@ -4218,7 +4218,7 @@
         </is>
       </c>
       <c r="J103" s="7" t="n">
-        <v>46281.44036814998</v>
+        <v>46281.44036814815</v>
       </c>
     </row>
     <row r="104">
@@ -4252,7 +4252,7 @@
         </is>
       </c>
       <c r="J104" s="7" t="n">
-        <v>46281.44036915404</v>
+        <v>46281.44036915509</v>
       </c>
     </row>
     <row r="105">
@@ -4286,7 +4286,7 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>46281.4403691543</v>
+        <v>46281.44036915509</v>
       </c>
     </row>
     <row r="106">
@@ -4320,7 +4320,7 @@
         </is>
       </c>
       <c r="J106" s="7" t="n">
-        <v>46281.44036915442</v>
+        <v>46281.44036915509</v>
       </c>
     </row>
     <row r="107">
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="J107" s="7" t="n">
-        <v>46281.44036915452</v>
+        <v>46281.44036915509</v>
       </c>
     </row>
     <row r="108">
@@ -4388,7 +4388,7 @@
         </is>
       </c>
       <c r="J108" s="7" t="n">
-        <v>46281.4403691546</v>
+        <v>46281.44036915509</v>
       </c>
     </row>
     <row r="109">
@@ -4422,7 +4422,7 @@
         </is>
       </c>
       <c r="J109" s="7" t="n">
-        <v>46281.44037853956</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="110">
@@ -4456,7 +4456,7 @@
         </is>
       </c>
       <c r="J110" s="7" t="n">
-        <v>46281.4403785399</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="111">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="J111" s="7" t="n">
-        <v>46281.44037854001</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="112">
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="J112" s="7" t="n">
-        <v>46281.4403785401</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="113">
@@ -4558,7 +4558,7 @@
         </is>
       </c>
       <c r="J113" s="7" t="n">
-        <v>46281.4403785402</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="114">
@@ -4592,7 +4592,7 @@
         </is>
       </c>
       <c r="J114" s="7" t="n">
-        <v>46281.44037854028</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="115">
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="J115" s="7" t="n">
-        <v>46281.44037854037</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="116">
@@ -4660,7 +4660,7 @@
         </is>
       </c>
       <c r="J116" s="7" t="n">
-        <v>46281.44037854045</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="117">
@@ -4694,7 +4694,7 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>46281.44037854054</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="118">
@@ -4728,7 +4728,7 @@
         </is>
       </c>
       <c r="J118" s="7" t="n">
-        <v>46281.44037854065</v>
+        <v>46281.44037854167</v>
       </c>
     </row>
     <row r="119">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="J119" s="7" t="n">
-        <v>46281.44038052983</v>
+        <v>46281.44038053241</v>
       </c>
     </row>
     <row r="120">
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="J120" s="7" t="n">
-        <v>46281.44038706453</v>
+        <v>46281.44038706018</v>
       </c>
     </row>
     <row r="121">
@@ -4830,7 +4830,7 @@
         </is>
       </c>
       <c r="J121" s="7" t="n">
-        <v>46281.44038706479</v>
+        <v>46281.44038706018</v>
       </c>
     </row>
     <row r="122">
@@ -4864,7 +4864,7 @@
         </is>
       </c>
       <c r="J122" s="7" t="n">
-        <v>46281.4403963969</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="123">
@@ -4906,7 +4906,7 @@
         </is>
       </c>
       <c r="J123" s="7" t="n">
-        <v>46281.44040258385</v>
+        <v>46281.44040258102</v>
       </c>
     </row>
     <row r="124">
@@ -4940,7 +4940,7 @@
         </is>
       </c>
       <c r="J124" s="7" t="n">
-        <v>46281.44039639729</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="125">
@@ -4974,7 +4974,7 @@
         </is>
       </c>
       <c r="J125" s="7" t="n">
-        <v>46281.44039639738</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="126">
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="J126" s="7" t="n">
-        <v>46281.44039639748</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="127">
@@ -5042,7 +5042,7 @@
         </is>
       </c>
       <c r="J127" s="7" t="n">
-        <v>46281.44039639757</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="128">
@@ -5076,7 +5076,7 @@
         </is>
       </c>
       <c r="J128" s="7" t="n">
-        <v>46281.44039639765</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="129">
@@ -5110,7 +5110,7 @@
         </is>
       </c>
       <c r="J129" s="7" t="n">
-        <v>46281.44039639775</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="130">
@@ -5144,7 +5144,7 @@
         </is>
       </c>
       <c r="J130" s="7" t="n">
-        <v>46281.44039639801</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="131">
@@ -5178,7 +5178,7 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>46281.44039639809</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="132">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>46281.44039639817</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="133">
@@ -5246,7 +5246,7 @@
         </is>
       </c>
       <c r="J133" s="7" t="n">
-        <v>46281.44039639826</v>
+        <v>46281.44039640046</v>
       </c>
     </row>
     <row r="134">
@@ -5280,7 +5280,7 @@
         </is>
       </c>
       <c r="J134" s="7" t="n">
-        <v>46281.44039837753</v>
+        <v>46281.44039837963</v>
       </c>
     </row>
     <row r="135">
@@ -5314,7 +5314,7 @@
         </is>
       </c>
       <c r="J135" s="7" t="n">
-        <v>46281.44040079451</v>
+        <v>46281.44040079861</v>
       </c>
     </row>
     <row r="136">
@@ -5348,7 +5348,7 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>46281.44041755493</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="137">
@@ -5382,7 +5382,7 @@
         </is>
       </c>
       <c r="J137" s="7" t="n">
-        <v>46281.44040079492</v>
+        <v>46281.44040079861</v>
       </c>
     </row>
     <row r="138">
@@ -5416,7 +5416,7 @@
         </is>
       </c>
       <c r="J138" s="7" t="n">
-        <v>46281.44040079501</v>
+        <v>46281.44040079861</v>
       </c>
     </row>
     <row r="139">
@@ -5450,7 +5450,7 @@
         </is>
       </c>
       <c r="J139" s="7" t="n">
-        <v>46281.44040258413</v>
+        <v>46281.44040258102</v>
       </c>
     </row>
     <row r="140">
@@ -5484,7 +5484,7 @@
         </is>
       </c>
       <c r="J140" s="7" t="n">
-        <v>46281.44040459942</v>
+        <v>46281.4404045949</v>
       </c>
     </row>
     <row r="141">
@@ -5518,7 +5518,7 @@
         </is>
       </c>
       <c r="J141" s="7" t="n">
-        <v>46281.44040551349</v>
+        <v>46281.44040550926</v>
       </c>
     </row>
     <row r="142">
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="J142" s="7" t="n">
-        <v>46281.44041263111</v>
+        <v>46281.44041262731</v>
       </c>
     </row>
     <row r="143">
@@ -5586,7 +5586,7 @@
         </is>
       </c>
       <c r="J143" s="7" t="n">
-        <v>46281.44041263137</v>
+        <v>46281.44041262731</v>
       </c>
     </row>
     <row r="144">
@@ -5620,7 +5620,7 @@
         </is>
       </c>
       <c r="J144" s="7" t="n">
-        <v>46281.44041263148</v>
+        <v>46281.44041262731</v>
       </c>
     </row>
     <row r="145">
@@ -5654,7 +5654,7 @@
         </is>
       </c>
       <c r="J145" s="7" t="n">
-        <v>46281.44041263157</v>
+        <v>46281.44041262731</v>
       </c>
     </row>
     <row r="146">
@@ -5688,7 +5688,7 @@
         </is>
       </c>
       <c r="J146" s="7" t="n">
-        <v>46281.44041356531</v>
+        <v>46281.44041356481</v>
       </c>
     </row>
     <row r="147">
@@ -5722,7 +5722,7 @@
         </is>
       </c>
       <c r="J147" s="7" t="n">
-        <v>46281.44041356556</v>
+        <v>46281.44041356481</v>
       </c>
     </row>
     <row r="148">
@@ -5756,7 +5756,7 @@
         </is>
       </c>
       <c r="J148" s="7" t="n">
-        <v>46281.44041356567</v>
+        <v>46281.44041356481</v>
       </c>
     </row>
     <row r="149">
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="J149" s="7" t="n">
-        <v>46281.44041755464</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="150">
@@ -5824,7 +5824,7 @@
         </is>
       </c>
       <c r="J150" s="7" t="n">
-        <v>46281.44041755512</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="151">
@@ -5858,7 +5858,7 @@
         </is>
       </c>
       <c r="J151" s="7" t="n">
-        <v>46281.44041755523</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="152">
@@ -5892,7 +5892,7 @@
         </is>
       </c>
       <c r="J152" s="7" t="n">
-        <v>46281.44041755541</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="153">
@@ -5926,7 +5926,7 @@
         </is>
       </c>
       <c r="J153" s="7" t="n">
-        <v>46281.44041755549</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="154">
@@ -5960,7 +5960,7 @@
         </is>
       </c>
       <c r="J154" s="7" t="n">
-        <v>46281.44041755566</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="155">
@@ -5994,7 +5994,7 @@
         </is>
       </c>
       <c r="J155" s="7" t="n">
-        <v>46281.44041755573</v>
+        <v>46281.44041755787</v>
       </c>
     </row>
     <row r="156">
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="J156" s="7" t="n">
-        <v>46281.44041854121</v>
+        <v>46281.44041854166</v>
       </c>
     </row>
     <row r="157">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="J157" s="7" t="n">
-        <v>46281.44041854141</v>
+        <v>46281.44041854166</v>
       </c>
     </row>
     <row r="158">
@@ -6096,7 +6096,7 @@
         </is>
       </c>
       <c r="J158" s="7" t="n">
-        <v>46281.44041854149</v>
+        <v>46281.44041854166</v>
       </c>
     </row>
     <row r="159">
@@ -6130,7 +6130,7 @@
         </is>
       </c>
       <c r="J159" s="7" t="n">
-        <v>46281.44041854158</v>
+        <v>46281.44041854166</v>
       </c>
     </row>
     <row r="160">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="J160" s="7" t="n">
-        <v>46281.44041952205</v>
+        <v>46281.44041952546</v>
       </c>
     </row>
     <row r="161">
@@ -6198,7 +6198,7 @@
         </is>
       </c>
       <c r="J161" s="7" t="n">
-        <v>46281.44041952214</v>
+        <v>46281.44041952546</v>
       </c>
     </row>
     <row r="162">
@@ -6232,7 +6232,7 @@
         </is>
       </c>
       <c r="J162" s="7" t="n">
-        <v>46281.44042136033</v>
+        <v>46281.44042136574</v>
       </c>
     </row>
     <row r="163">
@@ -6266,7 +6266,7 @@
         </is>
       </c>
       <c r="J163" s="7" t="n">
-        <v>46281.4404222552</v>
+        <v>46281.44042225694</v>
       </c>
     </row>
     <row r="164">
@@ -6296,11 +6296,11 @@
       <c r="H164" s="6" t="n"/>
       <c r="I164" t="inlineStr">
         <is>
-          <t>CA308662</t>
+          <t>CA316115</t>
         </is>
       </c>
       <c r="J164" s="7" t="n">
-        <v>46281.44036722396</v>
+        <v>46281.53116255045</v>
       </c>
     </row>
     <row r="165">
@@ -6334,7 +6334,7 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>46281.44036722426</v>
+        <v>46281.44036722223</v>
       </c>
     </row>
     <row r="166">
@@ -6368,7 +6368,7 @@
         </is>
       </c>
       <c r="J166" s="7" t="n">
-        <v>46281.44036722437</v>
+        <v>46281.44036722223</v>
       </c>
     </row>
     <row r="167">
@@ -6402,7 +6402,7 @@
         </is>
       </c>
       <c r="J167" s="7" t="n">
-        <v>46281.44036722447</v>
+        <v>46281.44036722223</v>
       </c>
     </row>
     <row r="168">
@@ -6436,7 +6436,7 @@
         </is>
       </c>
       <c r="J168" s="7" t="n">
-        <v>46281.44036722456</v>
+        <v>46281.44036722223</v>
       </c>
     </row>
     <row r="169">
@@ -6470,7 +6470,7 @@
         </is>
       </c>
       <c r="J169" s="7" t="n">
-        <v>46281.44036722464</v>
+        <v>46281.44036722223</v>
       </c>
     </row>
     <row r="170">
@@ -6504,7 +6504,7 @@
         </is>
       </c>
       <c r="J170" s="7" t="n">
-        <v>46281.44036722472</v>
+        <v>46281.44036722223</v>
       </c>
     </row>
     <row r="171">
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="J171" s="7" t="n">
-        <v>46281.4403672248</v>
+        <v>46281.44036722223</v>
       </c>
     </row>
     <row r="172">
@@ -6580,7 +6580,7 @@
         </is>
       </c>
       <c r="J172" s="7" t="n">
-        <v>46281.44044909777</v>
+        <v>46281.44044909722</v>
       </c>
     </row>
     <row r="173">
@@ -6613,7 +6613,7 @@
         </is>
       </c>
       <c r="J173" s="7" t="n">
-        <v>46281.44038268182</v>
+        <v>46281.44038268518</v>
       </c>
     </row>
     <row r="174">
@@ -6646,7 +6646,7 @@
         </is>
       </c>
       <c r="J174" s="7" t="n">
-        <v>46281.44038366416</v>
+        <v>46281.44038366898</v>
       </c>
     </row>
     <row r="175">
@@ -6679,7 +6679,7 @@
         </is>
       </c>
       <c r="J175" s="7" t="n">
-        <v>46281.44038366443</v>
+        <v>46281.44038366898</v>
       </c>
     </row>
     <row r="176">
@@ -6712,7 +6712,7 @@
         </is>
       </c>
       <c r="J176" s="7" t="n">
-        <v>46281.44039411465</v>
+        <v>46281.44039412037</v>
       </c>
     </row>
     <row r="177">
@@ -6745,7 +6745,7 @@
         </is>
       </c>
       <c r="J177" s="7" t="n">
-        <v>46281.44038465163</v>
+        <v>46281.44038465278</v>
       </c>
     </row>
     <row r="178">
@@ -6778,7 +6778,7 @@
         </is>
       </c>
       <c r="J178" s="7" t="n">
-        <v>46281.44038465223</v>
+        <v>46281.44038465278</v>
       </c>
     </row>
     <row r="179">
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="J179" s="7" t="n">
-        <v>46281.44044117146</v>
+        <v>46281.44044116898</v>
       </c>
     </row>
     <row r="180">
@@ -6853,7 +6853,73 @@
         </is>
       </c>
       <c r="J180" s="7" t="n">
-        <v>46281.44039113048</v>
+        <v>46281.44039113426</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>449886</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>NITRILE DIPPED GLOVES XL</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Chadwicks</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>CA316114</t>
+        </is>
+      </c>
+      <c r="J181" s="7" t="n">
+        <v>46281.5311615996</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>96335</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>CARBERY ATTIC TANK JACKET (PACK 10) AT44. AT58. AT45R, AT60R, AT80R</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>PACK</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Chadwicks</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>424.4</v>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>SX236186</t>
+        </is>
+      </c>
+      <c r="J182" s="7" t="n">
+        <v>46281.53116644685</v>
       </c>
     </row>
   </sheetData>
@@ -7065,7 +7131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1949"/>
+  <dimension ref="A1:H1951"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70153,6 +70219,66 @@
       <c r="G1949" t="inlineStr">
         <is>
           <t>SX235440</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>14/9/26</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>Chadwicks</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr">
+        <is>
+          <t>449886</t>
+        </is>
+      </c>
+      <c r="D1950" t="inlineStr">
+        <is>
+          <t>NITRILE DIPPED GLOVES XL</t>
+        </is>
+      </c>
+      <c r="F1950" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="G1950" t="inlineStr">
+        <is>
+          <t>CA316114</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>15/9/26</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>Chadwicks</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr">
+        <is>
+          <t>96335</t>
+        </is>
+      </c>
+      <c r="D1951" t="inlineStr">
+        <is>
+          <t>CARBERY ATTIC TANK JACKET (PACK 10) AT44. AT58. AT45R, AT60R, AT80R</t>
+        </is>
+      </c>
+      <c r="F1951" t="n">
+        <v>424.4</v>
+      </c>
+      <c r="G1951" t="inlineStr">
+        <is>
+          <t>SX236186</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated stoks with bales 100mm 60mm 20mm 10mm and add record for house f35kc82
</commit_message>
<xml_diff>
--- a/Chadwicks_FULL_INVOICES_TEST_NO_MATERIAL.xlsx
+++ b/Chadwicks_FULL_INVOICES_TEST_NO_MATERIAL.xlsx
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="J2" s="7" t="n">
-        <v>46281.68177670046</v>
+        <v>46282.69996056685</v>
       </c>
     </row>
     <row r="3">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>46281.68177670037</v>
+        <v>46282.69996056677</v>
       </c>
     </row>
     <row r="4">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="J4" s="7" t="n">
-        <v>46281.68177670028</v>
+        <v>46282.69996056668</v>
       </c>
     </row>
     <row r="5">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>46281.68177670017</v>
+        <v>46282.69996056658</v>
       </c>
     </row>
     <row r="6">
@@ -809,13 +809,13 @@
         <v>3.24</v>
       </c>
       <c r="F6" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>0.14</v>
+        <v>1.24</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.04516129032258065</v>
+        <v>0.62</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>46281.68177669989</v>
+        <v>46282.69996056629</v>
       </c>
     </row>
     <row r="7">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>46281.68177544424</v>
+        <v>46282.69995940327</v>
       </c>
     </row>
     <row r="8">
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>46281.68177451569</v>
+        <v>46282.69995856599</v>
       </c>
     </row>
     <row r="9">
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>46281.68177358562</v>
+        <v>46282.69995768993</v>
       </c>
     </row>
     <row r="10">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="J10" s="7" t="n">
-        <v>46281.68177358539</v>
+        <v>46282.69995768974</v>
       </c>
     </row>
     <row r="11">
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="J11" s="7" t="n">
-        <v>46281.68177358514</v>
+        <v>46282.69995768947</v>
       </c>
     </row>
     <row r="12">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="J12" s="7" t="n">
-        <v>46281.68177259171</v>
+        <v>46282.69995676125</v>
       </c>
     </row>
     <row r="13">
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>46281.68177169946</v>
+        <v>46282.69995593416</v>
       </c>
     </row>
     <row r="14">
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="J14" s="7" t="n">
-        <v>46281.68177077986</v>
+        <v>46282.69995509768</v>
       </c>
     </row>
     <row r="15">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="J15" s="7" t="n">
-        <v>46281.68177077957</v>
+        <v>46282.69995509737</v>
       </c>
     </row>
     <row r="16">
@@ -7142,7 +7142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1953"/>
+  <dimension ref="A1:H1955"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70354,6 +70354,72 @@
         <v>20.33</v>
       </c>
       <c r="G1953" t="inlineStr">
+        <is>
+          <t>SX235981</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>11/9/26</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr">
+        <is>
+          <t>Chadwicks</t>
+        </is>
+      </c>
+      <c r="C1954" t="inlineStr">
+        <is>
+          <t>22502</t>
+        </is>
+      </c>
+      <c r="D1954" t="inlineStr">
+        <is>
+          <t>BAUMIT PVC ANGLE (CORNER) BEAD WITH MESH 2.5M</t>
+        </is>
+      </c>
+      <c r="E1954" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1954" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="G1954" t="inlineStr">
+        <is>
+          <t>SX235981</t>
+        </is>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>11/9/26</t>
+        </is>
+      </c>
+      <c r="B1955" t="inlineStr">
+        <is>
+          <t>Chadwicks</t>
+        </is>
+      </c>
+      <c r="C1955" t="inlineStr">
+        <is>
+          <t>22502</t>
+        </is>
+      </c>
+      <c r="D1955" t="inlineStr">
+        <is>
+          <t>BAUMIT PVC ANGLE (CORNER) BEAD WITH MESH 2.5M</t>
+        </is>
+      </c>
+      <c r="E1955" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1955" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="G1955" t="inlineStr">
         <is>
           <t>SX235981</t>
         </is>

</xml_diff>